<commit_message>
v1.2.0 (build 3): add Brand category (10 categories, 1,200 words)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Multilingual_Vocabulary_1100.xlsx
+++ b/Multilingual_Vocabulary_1100.xlsx
@@ -1,26 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryopang/Documents/Claude Code/Project DUO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{148ACD86-E787-6543-BB8B-0700EDA79B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D990E6-E44C-9940-85F9-2FFF494F9FDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="780" windowWidth="28140" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$1</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5505" uniqueCount="2820">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6409" uniqueCount="3102">
   <si>
     <t>Category</t>
   </si>
@@ -8480,6 +8484,852 @@
   </si>
   <si>
     <t>松鼠鱖魚</t>
+  </si>
+  <si>
+    <t>Cantonese (Hong Kong)</t>
+  </si>
+  <si>
+    <t>Taiwan Chinese</t>
+  </si>
+  <si>
+    <t>Mainland Chinese</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>蘋果</t>
+  </si>
+  <si>
+    <t>苹果</t>
+  </si>
+  <si>
+    <t>Microsoft</t>
+  </si>
+  <si>
+    <t>微軟</t>
+  </si>
+  <si>
+    <t>微软</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>Google / 谷歌</t>
+  </si>
+  <si>
+    <t>谷歌</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>亞馬遜</t>
+  </si>
+  <si>
+    <t>亚马逊</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Facebook / 臉書</t>
+  </si>
+  <si>
+    <t>脸书</t>
+  </si>
+  <si>
+    <t>Netflix</t>
+  </si>
+  <si>
+    <t>Netflix / 網飛</t>
+  </si>
+  <si>
+    <t>网飞</t>
+  </si>
+  <si>
+    <t>Spotify</t>
+  </si>
+  <si>
+    <t>声田</t>
+  </si>
+  <si>
+    <t>Sony</t>
+  </si>
+  <si>
+    <t>Sony / 索尼</t>
+  </si>
+  <si>
+    <t>索尼</t>
+  </si>
+  <si>
+    <t>Samsung</t>
+  </si>
+  <si>
+    <t>三星</t>
+  </si>
+  <si>
+    <t>LG</t>
+  </si>
+  <si>
+    <t>Panasonic</t>
+  </si>
+  <si>
+    <t>樂聲</t>
+  </si>
+  <si>
+    <t>Panasonic / 國際牌</t>
+  </si>
+  <si>
+    <t>松下</t>
+  </si>
+  <si>
+    <t>Dell</t>
+  </si>
+  <si>
+    <t>Dell / 戴爾</t>
+  </si>
+  <si>
+    <t>戴尔</t>
+  </si>
+  <si>
+    <t>HP</t>
+  </si>
+  <si>
+    <t>HP / 惠普</t>
+  </si>
+  <si>
+    <t>惠普</t>
+  </si>
+  <si>
+    <t>Lenovo</t>
+  </si>
+  <si>
+    <t>Lenovo / 聯想</t>
+  </si>
+  <si>
+    <t>联想</t>
+  </si>
+  <si>
+    <t>Asus</t>
+  </si>
+  <si>
+    <t>Asus / 華碩</t>
+  </si>
+  <si>
+    <t>华硕</t>
+  </si>
+  <si>
+    <t>Acer</t>
+  </si>
+  <si>
+    <t>Acer / 宏碁</t>
+  </si>
+  <si>
+    <t>宏碁</t>
+  </si>
+  <si>
+    <t>Intel</t>
+  </si>
+  <si>
+    <t>Intel / 英特爾</t>
+  </si>
+  <si>
+    <t>英特尔</t>
+  </si>
+  <si>
+    <t>AMD</t>
+  </si>
+  <si>
+    <t>AMD / 超微</t>
+  </si>
+  <si>
+    <t>超威</t>
+  </si>
+  <si>
+    <t>Nvidia</t>
+  </si>
+  <si>
+    <t>Nvidia / 輝達</t>
+  </si>
+  <si>
+    <t>英伟达</t>
+  </si>
+  <si>
+    <t>Nintendo</t>
+  </si>
+  <si>
+    <t>任天堂</t>
+  </si>
+  <si>
+    <t>Toyota</t>
+  </si>
+  <si>
+    <t>豐田</t>
+  </si>
+  <si>
+    <t>丰田</t>
+  </si>
+  <si>
+    <t>Honda</t>
+  </si>
+  <si>
+    <t>本田</t>
+  </si>
+  <si>
+    <t>Nissan</t>
+  </si>
+  <si>
+    <t>日產</t>
+  </si>
+  <si>
+    <t>日产</t>
+  </si>
+  <si>
+    <t>BMW</t>
+  </si>
+  <si>
+    <t>寶馬</t>
+  </si>
+  <si>
+    <t>BMW / 寶馬</t>
+  </si>
+  <si>
+    <t>宝马</t>
+  </si>
+  <si>
+    <t>Mercedes-Benz</t>
+  </si>
+  <si>
+    <t>平治</t>
+  </si>
+  <si>
+    <t>賓士</t>
+  </si>
+  <si>
+    <t>奔驰</t>
+  </si>
+  <si>
+    <t>Volkswagen</t>
+  </si>
+  <si>
+    <t>福士</t>
+  </si>
+  <si>
+    <t>福斯</t>
+  </si>
+  <si>
+    <t>大众</t>
+  </si>
+  <si>
+    <t>Porsche</t>
+  </si>
+  <si>
+    <t>保時捷</t>
+  </si>
+  <si>
+    <t>保时捷</t>
+  </si>
+  <si>
+    <t>Audi</t>
+  </si>
+  <si>
+    <t>奧迪</t>
+  </si>
+  <si>
+    <t>奥迪</t>
+  </si>
+  <si>
+    <t>Lexus</t>
+  </si>
+  <si>
+    <t>凌志</t>
+  </si>
+  <si>
+    <t>Lexus / 凌志</t>
+  </si>
+  <si>
+    <t>雷克萨斯</t>
+  </si>
+  <si>
+    <t>Land Rover</t>
+  </si>
+  <si>
+    <t>越野路華</t>
+  </si>
+  <si>
+    <t>Land Rover / 荒原路華</t>
+  </si>
+  <si>
+    <t>路虎</t>
+  </si>
+  <si>
+    <t>Jaguar</t>
+  </si>
+  <si>
+    <t>積架</t>
+  </si>
+  <si>
+    <t>Jaguar / 捷豹</t>
+  </si>
+  <si>
+    <t>捷豹</t>
+  </si>
+  <si>
+    <t>Mazda</t>
+  </si>
+  <si>
+    <t>萬事得</t>
+  </si>
+  <si>
+    <t>Mazda / 馬自達</t>
+  </si>
+  <si>
+    <t>马自达</t>
+  </si>
+  <si>
+    <t>Subaru</t>
+  </si>
+  <si>
+    <t>富士</t>
+  </si>
+  <si>
+    <t>Subaru / 速霸陸</t>
+  </si>
+  <si>
+    <t>斯巴鲁</t>
+  </si>
+  <si>
+    <t>Volvo</t>
+  </si>
+  <si>
+    <t>富豪</t>
+  </si>
+  <si>
+    <t>Volvo / 富豪</t>
+  </si>
+  <si>
+    <t>沃尔沃</t>
+  </si>
+  <si>
+    <t>Ford</t>
+  </si>
+  <si>
+    <t>福特</t>
+  </si>
+  <si>
+    <t>McDonald's</t>
+  </si>
+  <si>
+    <t>麥當勞</t>
+  </si>
+  <si>
+    <t>麦当劳</t>
+  </si>
+  <si>
+    <t>KFC</t>
+  </si>
+  <si>
+    <t>肯德基</t>
+  </si>
+  <si>
+    <t>Starbucks</t>
+  </si>
+  <si>
+    <t>星巴克</t>
+  </si>
+  <si>
+    <t>Burger King</t>
+  </si>
+  <si>
+    <t>漢堡王</t>
+  </si>
+  <si>
+    <t>汉堡王</t>
+  </si>
+  <si>
+    <t>Pizza Hut</t>
+  </si>
+  <si>
+    <t>必勝客</t>
+  </si>
+  <si>
+    <t>必胜客</t>
+  </si>
+  <si>
+    <t>Subway</t>
+  </si>
+  <si>
+    <t>Subway / 賽百味</t>
+  </si>
+  <si>
+    <t>赛百味</t>
+  </si>
+  <si>
+    <t>Coca-Cola</t>
+  </si>
+  <si>
+    <t>可口可樂</t>
+  </si>
+  <si>
+    <t>可口可乐</t>
+  </si>
+  <si>
+    <t>Pepsi</t>
+  </si>
+  <si>
+    <t>百事可樂</t>
+  </si>
+  <si>
+    <t>百事可乐</t>
+  </si>
+  <si>
+    <t>Sprite</t>
+  </si>
+  <si>
+    <t>Fanta</t>
+  </si>
+  <si>
+    <t>芬达</t>
+  </si>
+  <si>
+    <t>Lipton</t>
+  </si>
+  <si>
+    <t>立頓</t>
+  </si>
+  <si>
+    <t>立顿</t>
+  </si>
+  <si>
+    <t>Nestle</t>
+  </si>
+  <si>
+    <t>雀巢</t>
+  </si>
+  <si>
+    <t>Heinz</t>
+  </si>
+  <si>
+    <t>亨氏</t>
+  </si>
+  <si>
+    <t>Kellogg's</t>
+  </si>
+  <si>
+    <t>家樂氏</t>
+  </si>
+  <si>
+    <t>家乐氏</t>
+  </si>
+  <si>
+    <t>Lay's</t>
+  </si>
+  <si>
+    <t>樂事</t>
+  </si>
+  <si>
+    <t>乐事</t>
+  </si>
+  <si>
+    <t>M&amp;M's</t>
+  </si>
+  <si>
+    <t>Snickers</t>
+  </si>
+  <si>
+    <t>士力架</t>
+  </si>
+  <si>
+    <t>Skittles</t>
+  </si>
+  <si>
+    <t>彩虹糖</t>
+  </si>
+  <si>
+    <t>Oreo</t>
+  </si>
+  <si>
+    <t>奧利奧</t>
+  </si>
+  <si>
+    <t>奥利奥</t>
+  </si>
+  <si>
+    <t>Marriott</t>
+  </si>
+  <si>
+    <t>萬豪</t>
+  </si>
+  <si>
+    <t>万豪</t>
+  </si>
+  <si>
+    <t>Red Bull</t>
+  </si>
+  <si>
+    <t>紅牛</t>
+  </si>
+  <si>
+    <t>红牛</t>
+  </si>
+  <si>
+    <t>Heineken</t>
+  </si>
+  <si>
+    <t>喜力</t>
+  </si>
+  <si>
+    <t>海尼根</t>
+  </si>
+  <si>
+    <t>Carlsberg</t>
+  </si>
+  <si>
+    <t>嘉士伯</t>
+  </si>
+  <si>
+    <t>Guinness</t>
+  </si>
+  <si>
+    <t>健力士</t>
+  </si>
+  <si>
+    <t>Evian</t>
+  </si>
+  <si>
+    <t>依雲</t>
+  </si>
+  <si>
+    <t>愛維養</t>
+  </si>
+  <si>
+    <t>依云</t>
+  </si>
+  <si>
+    <t>Pampers</t>
+  </si>
+  <si>
+    <t>幫寶適</t>
+  </si>
+  <si>
+    <t>帮宝适</t>
+  </si>
+  <si>
+    <t>多芬</t>
+  </si>
+  <si>
+    <t>Pantene</t>
+  </si>
+  <si>
+    <t>潘婷</t>
+  </si>
+  <si>
+    <t>Head &amp; Shoulders</t>
+  </si>
+  <si>
+    <t>海飛絲</t>
+  </si>
+  <si>
+    <t>海倫仙度絲</t>
+  </si>
+  <si>
+    <t>海飞丝</t>
+  </si>
+  <si>
+    <t>Crest</t>
+  </si>
+  <si>
+    <t>佳潔士</t>
+  </si>
+  <si>
+    <t>固齒佳</t>
+  </si>
+  <si>
+    <t>佳洁士</t>
+  </si>
+  <si>
+    <t>Colgate</t>
+  </si>
+  <si>
+    <t>高露潔</t>
+  </si>
+  <si>
+    <t>高露洁</t>
+  </si>
+  <si>
+    <t>Gillette</t>
+  </si>
+  <si>
+    <t>吉列</t>
+  </si>
+  <si>
+    <t>L'Oréal</t>
+  </si>
+  <si>
+    <t>巴黎歐萊雅</t>
+  </si>
+  <si>
+    <t>巴黎萊雅</t>
+  </si>
+  <si>
+    <t>巴黎欧莱雅</t>
+  </si>
+  <si>
+    <t>Darlie</t>
+  </si>
+  <si>
+    <t>好來</t>
+  </si>
+  <si>
+    <t>好来</t>
+  </si>
+  <si>
+    <t>Shiseido</t>
+  </si>
+  <si>
+    <t>資生堂</t>
+  </si>
+  <si>
+    <t>资生堂</t>
+  </si>
+  <si>
+    <t>Nike</t>
+  </si>
+  <si>
+    <t>Nike / 耐吉</t>
+  </si>
+  <si>
+    <t>耐克</t>
+  </si>
+  <si>
+    <t>Adidas</t>
+  </si>
+  <si>
+    <t>Adidas / 愛迪達</t>
+  </si>
+  <si>
+    <t>阿迪达斯</t>
+  </si>
+  <si>
+    <t>Puma</t>
+  </si>
+  <si>
+    <t>Puma / 彪馬</t>
+  </si>
+  <si>
+    <t>彪马</t>
+  </si>
+  <si>
+    <t>Zara</t>
+  </si>
+  <si>
+    <t>萨拉</t>
+  </si>
+  <si>
+    <t>H&amp;M</t>
+  </si>
+  <si>
+    <t>Uniqlo</t>
+  </si>
+  <si>
+    <t>Uniqlo / 優衣庫</t>
+  </si>
+  <si>
+    <t>优衣库</t>
+  </si>
+  <si>
+    <t>Levi's</t>
+  </si>
+  <si>
+    <t>李维斯</t>
+  </si>
+  <si>
+    <t>Chanel</t>
+  </si>
+  <si>
+    <t>香奈兒</t>
+  </si>
+  <si>
+    <t>香奈儿</t>
+  </si>
+  <si>
+    <t>Hermes</t>
+  </si>
+  <si>
+    <t>愛馬仕</t>
+  </si>
+  <si>
+    <t>爱马仕</t>
+  </si>
+  <si>
+    <t>Louis Vuitton</t>
+  </si>
+  <si>
+    <t>LV / 路易威登</t>
+  </si>
+  <si>
+    <t>Gucci</t>
+  </si>
+  <si>
+    <t>Gucci / 古馳</t>
+  </si>
+  <si>
+    <t>古驰</t>
+  </si>
+  <si>
+    <t>Prada</t>
+  </si>
+  <si>
+    <t>Prada / 普拉達</t>
+  </si>
+  <si>
+    <t>普拉达</t>
+  </si>
+  <si>
+    <t>Burberry</t>
+  </si>
+  <si>
+    <t>Burberry / 巴寶莉</t>
+  </si>
+  <si>
+    <t>博柏利</t>
+  </si>
+  <si>
+    <t>Rolex</t>
+  </si>
+  <si>
+    <t>勞力士</t>
+  </si>
+  <si>
+    <t>劳力士</t>
+  </si>
+  <si>
+    <t>Cartier</t>
+  </si>
+  <si>
+    <t>卡地亞</t>
+  </si>
+  <si>
+    <t>卡地亚</t>
+  </si>
+  <si>
+    <t>Disney</t>
+  </si>
+  <si>
+    <t>迪士尼</t>
+  </si>
+  <si>
+    <t>Marvel</t>
+  </si>
+  <si>
+    <t>漫威</t>
+  </si>
+  <si>
+    <t>Warner Bros.</t>
+  </si>
+  <si>
+    <t>華納兄弟</t>
+  </si>
+  <si>
+    <t>华纳兄弟</t>
+  </si>
+  <si>
+    <t>Universal Studios</t>
+  </si>
+  <si>
+    <t>環球影城</t>
+  </si>
+  <si>
+    <t>环球影城</t>
+  </si>
+  <si>
+    <t>Lego</t>
+  </si>
+  <si>
+    <t>樂高</t>
+  </si>
+  <si>
+    <t>乐高</t>
+  </si>
+  <si>
+    <t>Hasbro</t>
+  </si>
+  <si>
+    <t>孩之寶</t>
+  </si>
+  <si>
+    <t>孩之宝</t>
+  </si>
+  <si>
+    <t>IKEA</t>
+  </si>
+  <si>
+    <t>宜家傢俬</t>
+  </si>
+  <si>
+    <t>IKEA / 宜家家居</t>
+  </si>
+  <si>
+    <t>宜家</t>
+  </si>
+  <si>
+    <t>Visa</t>
+  </si>
+  <si>
+    <t>Mastercard</t>
+  </si>
+  <si>
+    <t>Mastercard / 萬事達卡</t>
+  </si>
+  <si>
+    <t>万事达卡</t>
+  </si>
+  <si>
+    <t>American Express</t>
+  </si>
+  <si>
+    <t>美國運通</t>
+  </si>
+  <si>
+    <t>美国运通</t>
+  </si>
+  <si>
+    <t>PayPal</t>
+  </si>
+  <si>
+    <t>贝宝</t>
+  </si>
+  <si>
+    <t>eBay</t>
+  </si>
+  <si>
+    <t>易趣</t>
+  </si>
+  <si>
+    <t>Alibaba</t>
+  </si>
+  <si>
+    <t>阿里巴巴</t>
+  </si>
+  <si>
+    <t>Tencent</t>
+  </si>
+  <si>
+    <t>騰訊</t>
+  </si>
+  <si>
+    <t>腾讯</t>
+  </si>
+  <si>
+    <t>Baidu</t>
+  </si>
+  <si>
+    <t>百度</t>
+  </si>
+  <si>
+    <t>Brand</t>
   </si>
 </sst>
 </file>
@@ -8847,7 +9697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1101"/>
+  <dimension ref="A1:E1201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -27573,6 +28423,3131 @@
         <v>2165</v>
       </c>
     </row>
+    <row r="1102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1102" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1102" t="s">
+        <v>2823</v>
+      </c>
+      <c r="C1102" t="s">
+        <v>2824</v>
+      </c>
+      <c r="D1102" t="s">
+        <v>2824</v>
+      </c>
+      <c r="E1102" t="s">
+        <v>2825</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1103" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1103" t="s">
+        <v>2826</v>
+      </c>
+      <c r="C1103" t="s">
+        <v>2827</v>
+      </c>
+      <c r="D1103" t="s">
+        <v>2827</v>
+      </c>
+      <c r="E1103" t="s">
+        <v>2828</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1104" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1104" t="s">
+        <v>2829</v>
+      </c>
+      <c r="C1104" t="s">
+        <v>2829</v>
+      </c>
+      <c r="D1104" t="s">
+        <v>2830</v>
+      </c>
+      <c r="E1104" t="s">
+        <v>2831</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1105" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1105" t="s">
+        <v>2832</v>
+      </c>
+      <c r="C1105" t="s">
+        <v>2833</v>
+      </c>
+      <c r="D1105" t="s">
+        <v>2833</v>
+      </c>
+      <c r="E1105" t="s">
+        <v>2834</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1106" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1106" t="s">
+        <v>2835</v>
+      </c>
+      <c r="C1106" t="s">
+        <v>2835</v>
+      </c>
+      <c r="D1106" t="s">
+        <v>2836</v>
+      </c>
+      <c r="E1106" t="s">
+        <v>2837</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1107" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1107" t="s">
+        <v>2838</v>
+      </c>
+      <c r="C1107" t="s">
+        <v>2838</v>
+      </c>
+      <c r="D1107" t="s">
+        <v>2839</v>
+      </c>
+      <c r="E1107" t="s">
+        <v>2840</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1108" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1108" t="s">
+        <v>2841</v>
+      </c>
+      <c r="C1108" t="s">
+        <v>2841</v>
+      </c>
+      <c r="D1108" t="s">
+        <v>2841</v>
+      </c>
+      <c r="E1108" t="s">
+        <v>2842</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1109" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1109" t="s">
+        <v>2843</v>
+      </c>
+      <c r="C1109" t="s">
+        <v>2844</v>
+      </c>
+      <c r="D1109" t="s">
+        <v>2844</v>
+      </c>
+      <c r="E1109" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1110" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1110" t="s">
+        <v>2846</v>
+      </c>
+      <c r="C1110" t="s">
+        <v>2847</v>
+      </c>
+      <c r="D1110" t="s">
+        <v>2847</v>
+      </c>
+      <c r="E1110" t="s">
+        <v>2847</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1111" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1111" t="s">
+        <v>2848</v>
+      </c>
+      <c r="C1111" t="s">
+        <v>2848</v>
+      </c>
+      <c r="D1111" t="s">
+        <v>2848</v>
+      </c>
+      <c r="E1111" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1112" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1112" t="s">
+        <v>2849</v>
+      </c>
+      <c r="C1112" t="s">
+        <v>2850</v>
+      </c>
+      <c r="D1112" t="s">
+        <v>2851</v>
+      </c>
+      <c r="E1112" t="s">
+        <v>2852</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1113" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1113" t="s">
+        <v>2853</v>
+      </c>
+      <c r="C1113" t="s">
+        <v>2853</v>
+      </c>
+      <c r="D1113" t="s">
+        <v>2854</v>
+      </c>
+      <c r="E1113" t="s">
+        <v>2855</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1114" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1114" t="s">
+        <v>2856</v>
+      </c>
+      <c r="C1114" t="s">
+        <v>2856</v>
+      </c>
+      <c r="D1114" t="s">
+        <v>2857</v>
+      </c>
+      <c r="E1114" t="s">
+        <v>2858</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1115" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1115" t="s">
+        <v>2859</v>
+      </c>
+      <c r="C1115" t="s">
+        <v>2859</v>
+      </c>
+      <c r="D1115" t="s">
+        <v>2860</v>
+      </c>
+      <c r="E1115" t="s">
+        <v>2861</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1116" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1116" t="s">
+        <v>2862</v>
+      </c>
+      <c r="C1116" t="s">
+        <v>2862</v>
+      </c>
+      <c r="D1116" t="s">
+        <v>2863</v>
+      </c>
+      <c r="E1116" t="s">
+        <v>2864</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1117" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1117" t="s">
+        <v>2865</v>
+      </c>
+      <c r="C1117" t="s">
+        <v>2865</v>
+      </c>
+      <c r="D1117" t="s">
+        <v>2866</v>
+      </c>
+      <c r="E1117" t="s">
+        <v>2867</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1118" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1118" t="s">
+        <v>2868</v>
+      </c>
+      <c r="C1118" t="s">
+        <v>2868</v>
+      </c>
+      <c r="D1118" t="s">
+        <v>2869</v>
+      </c>
+      <c r="E1118" t="s">
+        <v>2870</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1119" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1119" t="s">
+        <v>2871</v>
+      </c>
+      <c r="C1119" t="s">
+        <v>2871</v>
+      </c>
+      <c r="D1119" t="s">
+        <v>2872</v>
+      </c>
+      <c r="E1119" t="s">
+        <v>2873</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1120" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1120" t="s">
+        <v>2874</v>
+      </c>
+      <c r="C1120" t="s">
+        <v>2874</v>
+      </c>
+      <c r="D1120" t="s">
+        <v>2875</v>
+      </c>
+      <c r="E1120" t="s">
+        <v>2876</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1121" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1121" t="s">
+        <v>2877</v>
+      </c>
+      <c r="C1121" t="s">
+        <v>2878</v>
+      </c>
+      <c r="D1121" t="s">
+        <v>2878</v>
+      </c>
+      <c r="E1121" t="s">
+        <v>2878</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1122" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1122" t="s">
+        <v>2879</v>
+      </c>
+      <c r="C1122" t="s">
+        <v>2880</v>
+      </c>
+      <c r="D1122" t="s">
+        <v>2880</v>
+      </c>
+      <c r="E1122" t="s">
+        <v>2881</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1123" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1123" t="s">
+        <v>2882</v>
+      </c>
+      <c r="C1123" t="s">
+        <v>2883</v>
+      </c>
+      <c r="D1123" t="s">
+        <v>2883</v>
+      </c>
+      <c r="E1123" t="s">
+        <v>2883</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1124" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1124" t="s">
+        <v>2884</v>
+      </c>
+      <c r="C1124" t="s">
+        <v>2885</v>
+      </c>
+      <c r="D1124" t="s">
+        <v>2885</v>
+      </c>
+      <c r="E1124" t="s">
+        <v>2886</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1125" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1125" t="s">
+        <v>2887</v>
+      </c>
+      <c r="C1125" t="s">
+        <v>2888</v>
+      </c>
+      <c r="D1125" t="s">
+        <v>2889</v>
+      </c>
+      <c r="E1125" t="s">
+        <v>2890</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1126" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1126" t="s">
+        <v>2891</v>
+      </c>
+      <c r="C1126" t="s">
+        <v>2892</v>
+      </c>
+      <c r="D1126" t="s">
+        <v>2893</v>
+      </c>
+      <c r="E1126" t="s">
+        <v>2894</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1127" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1127" t="s">
+        <v>2895</v>
+      </c>
+      <c r="C1127" t="s">
+        <v>2896</v>
+      </c>
+      <c r="D1127" t="s">
+        <v>2897</v>
+      </c>
+      <c r="E1127" t="s">
+        <v>2898</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1128" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1128" t="s">
+        <v>2899</v>
+      </c>
+      <c r="C1128" t="s">
+        <v>2900</v>
+      </c>
+      <c r="D1128" t="s">
+        <v>2900</v>
+      </c>
+      <c r="E1128" t="s">
+        <v>2901</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1129" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1129" t="s">
+        <v>2902</v>
+      </c>
+      <c r="C1129" t="s">
+        <v>2903</v>
+      </c>
+      <c r="D1129" t="s">
+        <v>2903</v>
+      </c>
+      <c r="E1129" t="s">
+        <v>2904</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1130" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1130" t="s">
+        <v>2905</v>
+      </c>
+      <c r="C1130" t="s">
+        <v>2906</v>
+      </c>
+      <c r="D1130" t="s">
+        <v>2907</v>
+      </c>
+      <c r="E1130" t="s">
+        <v>2908</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1131" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1131" t="s">
+        <v>2909</v>
+      </c>
+      <c r="C1131" t="s">
+        <v>2910</v>
+      </c>
+      <c r="D1131" t="s">
+        <v>2911</v>
+      </c>
+      <c r="E1131" t="s">
+        <v>2912</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1132" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1132" t="s">
+        <v>2913</v>
+      </c>
+      <c r="C1132" t="s">
+        <v>2914</v>
+      </c>
+      <c r="D1132" t="s">
+        <v>2915</v>
+      </c>
+      <c r="E1132" t="s">
+        <v>2916</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1133" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1133" t="s">
+        <v>2917</v>
+      </c>
+      <c r="C1133" t="s">
+        <v>2918</v>
+      </c>
+      <c r="D1133" t="s">
+        <v>2919</v>
+      </c>
+      <c r="E1133" t="s">
+        <v>2920</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1134" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1134" t="s">
+        <v>2921</v>
+      </c>
+      <c r="C1134" t="s">
+        <v>2922</v>
+      </c>
+      <c r="D1134" t="s">
+        <v>2923</v>
+      </c>
+      <c r="E1134" t="s">
+        <v>2924</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1135" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1135" t="s">
+        <v>2925</v>
+      </c>
+      <c r="C1135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="D1135" t="s">
+        <v>2927</v>
+      </c>
+      <c r="E1135" t="s">
+        <v>2928</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1136" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1136" t="s">
+        <v>2929</v>
+      </c>
+      <c r="C1136" t="s">
+        <v>2930</v>
+      </c>
+      <c r="D1136" t="s">
+        <v>2930</v>
+      </c>
+      <c r="E1136" t="s">
+        <v>2930</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1137" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1137" t="s">
+        <v>2931</v>
+      </c>
+      <c r="C1137" t="s">
+        <v>2932</v>
+      </c>
+      <c r="D1137" t="s">
+        <v>2932</v>
+      </c>
+      <c r="E1137" t="s">
+        <v>2933</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1138" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1138" t="s">
+        <v>2934</v>
+      </c>
+      <c r="C1138" t="s">
+        <v>2935</v>
+      </c>
+      <c r="D1138" t="s">
+        <v>2935</v>
+      </c>
+      <c r="E1138" t="s">
+        <v>2935</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1139" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1139" t="s">
+        <v>2936</v>
+      </c>
+      <c r="C1139" t="s">
+        <v>2937</v>
+      </c>
+      <c r="D1139" t="s">
+        <v>2937</v>
+      </c>
+      <c r="E1139" t="s">
+        <v>2937</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1140" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1140" t="s">
+        <v>2938</v>
+      </c>
+      <c r="C1140" t="s">
+        <v>2939</v>
+      </c>
+      <c r="D1140" t="s">
+        <v>2939</v>
+      </c>
+      <c r="E1140" t="s">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1141" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1141" t="s">
+        <v>2941</v>
+      </c>
+      <c r="C1141" t="s">
+        <v>2942</v>
+      </c>
+      <c r="D1141" t="s">
+        <v>2942</v>
+      </c>
+      <c r="E1141" t="s">
+        <v>2943</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1142" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1142" t="s">
+        <v>2944</v>
+      </c>
+      <c r="C1142" t="s">
+        <v>2944</v>
+      </c>
+      <c r="D1142" t="s">
+        <v>2945</v>
+      </c>
+      <c r="E1142" t="s">
+        <v>2946</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1143" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1143" t="s">
+        <v>2947</v>
+      </c>
+      <c r="C1143" t="s">
+        <v>2948</v>
+      </c>
+      <c r="D1143" t="s">
+        <v>2948</v>
+      </c>
+      <c r="E1143" t="s">
+        <v>2949</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1144" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1144" t="s">
+        <v>2950</v>
+      </c>
+      <c r="C1144" t="s">
+        <v>2951</v>
+      </c>
+      <c r="D1144" t="s">
+        <v>2951</v>
+      </c>
+      <c r="E1144" t="s">
+        <v>2952</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1145" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1145" t="s">
+        <v>2953</v>
+      </c>
+      <c r="C1145" t="s">
+        <v>1753</v>
+      </c>
+      <c r="D1145" t="s">
+        <v>1753</v>
+      </c>
+      <c r="E1145" t="s">
+        <v>1753</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1146" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1146" t="s">
+        <v>2954</v>
+      </c>
+      <c r="C1146" t="s">
+        <v>1756</v>
+      </c>
+      <c r="D1146" t="s">
+        <v>1756</v>
+      </c>
+      <c r="E1146" t="s">
+        <v>2955</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1147" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1147" t="s">
+        <v>2956</v>
+      </c>
+      <c r="C1147" t="s">
+        <v>2957</v>
+      </c>
+      <c r="D1147" t="s">
+        <v>2957</v>
+      </c>
+      <c r="E1147" t="s">
+        <v>2958</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1148" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1148" t="s">
+        <v>2959</v>
+      </c>
+      <c r="C1148" t="s">
+        <v>2960</v>
+      </c>
+      <c r="D1148" t="s">
+        <v>2960</v>
+      </c>
+      <c r="E1148" t="s">
+        <v>2960</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1149" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1149" t="s">
+        <v>2961</v>
+      </c>
+      <c r="C1149" t="s">
+        <v>2962</v>
+      </c>
+      <c r="D1149" t="s">
+        <v>2962</v>
+      </c>
+      <c r="E1149" t="s">
+        <v>2962</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1150" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1150" t="s">
+        <v>2963</v>
+      </c>
+      <c r="C1150" t="s">
+        <v>2964</v>
+      </c>
+      <c r="D1150" t="s">
+        <v>2964</v>
+      </c>
+      <c r="E1150" t="s">
+        <v>2965</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1151" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1151" t="s">
+        <v>2966</v>
+      </c>
+      <c r="C1151" t="s">
+        <v>2967</v>
+      </c>
+      <c r="D1151" t="s">
+        <v>2967</v>
+      </c>
+      <c r="E1151" t="s">
+        <v>2968</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1152" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1152" t="s">
+        <v>2969</v>
+      </c>
+      <c r="C1152" t="s">
+        <v>2969</v>
+      </c>
+      <c r="D1152" t="s">
+        <v>2969</v>
+      </c>
+      <c r="E1152" t="s">
+        <v>2969</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1153" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1153" t="s">
+        <v>2970</v>
+      </c>
+      <c r="C1153" t="s">
+        <v>2971</v>
+      </c>
+      <c r="D1153" t="s">
+        <v>2971</v>
+      </c>
+      <c r="E1153" t="s">
+        <v>2971</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1154" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1154" t="s">
+        <v>2972</v>
+      </c>
+      <c r="C1154" t="s">
+        <v>2973</v>
+      </c>
+      <c r="D1154" t="s">
+        <v>2973</v>
+      </c>
+      <c r="E1154" t="s">
+        <v>2973</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1155" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1155" t="s">
+        <v>2974</v>
+      </c>
+      <c r="C1155" t="s">
+        <v>2975</v>
+      </c>
+      <c r="D1155" t="s">
+        <v>2975</v>
+      </c>
+      <c r="E1155" t="s">
+        <v>2976</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1156" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1156" t="s">
+        <v>2977</v>
+      </c>
+      <c r="C1156" t="s">
+        <v>2978</v>
+      </c>
+      <c r="D1156" t="s">
+        <v>2978</v>
+      </c>
+      <c r="E1156" t="s">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1157" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1157" t="s">
+        <v>2980</v>
+      </c>
+      <c r="C1157" t="s">
+        <v>2981</v>
+      </c>
+      <c r="D1157" t="s">
+        <v>2981</v>
+      </c>
+      <c r="E1157" t="s">
+        <v>2982</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1158" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1158" t="s">
+        <v>2983</v>
+      </c>
+      <c r="C1158" t="s">
+        <v>2984</v>
+      </c>
+      <c r="D1158" t="s">
+        <v>2985</v>
+      </c>
+      <c r="E1158" t="s">
+        <v>2984</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1159" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1159" t="s">
+        <v>2986</v>
+      </c>
+      <c r="C1159" t="s">
+        <v>2987</v>
+      </c>
+      <c r="D1159" t="s">
+        <v>2987</v>
+      </c>
+      <c r="E1159" t="s">
+        <v>2987</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1160" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1160" t="s">
+        <v>2988</v>
+      </c>
+      <c r="C1160" t="s">
+        <v>2989</v>
+      </c>
+      <c r="D1160" t="s">
+        <v>2989</v>
+      </c>
+      <c r="E1160" t="s">
+        <v>2989</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1161" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1161" t="s">
+        <v>2990</v>
+      </c>
+      <c r="C1161" t="s">
+        <v>2991</v>
+      </c>
+      <c r="D1161" t="s">
+        <v>2992</v>
+      </c>
+      <c r="E1161" t="s">
+        <v>2993</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1162" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1162" t="s">
+        <v>2994</v>
+      </c>
+      <c r="C1162" t="s">
+        <v>2995</v>
+      </c>
+      <c r="D1162" t="s">
+        <v>2995</v>
+      </c>
+      <c r="E1162" t="s">
+        <v>2996</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1163" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1163" t="s">
+        <v>583</v>
+      </c>
+      <c r="C1163" t="s">
+        <v>2997</v>
+      </c>
+      <c r="D1163" t="s">
+        <v>2997</v>
+      </c>
+      <c r="E1163" t="s">
+        <v>2997</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1164" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1164" t="s">
+        <v>2998</v>
+      </c>
+      <c r="C1164" t="s">
+        <v>2999</v>
+      </c>
+      <c r="D1164" t="s">
+        <v>2999</v>
+      </c>
+      <c r="E1164" t="s">
+        <v>2999</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1165" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1165" t="s">
+        <v>3000</v>
+      </c>
+      <c r="C1165" t="s">
+        <v>3001</v>
+      </c>
+      <c r="D1165" t="s">
+        <v>3002</v>
+      </c>
+      <c r="E1165" t="s">
+        <v>3003</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1166" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1166" t="s">
+        <v>3004</v>
+      </c>
+      <c r="C1166" t="s">
+        <v>3005</v>
+      </c>
+      <c r="D1166" t="s">
+        <v>3006</v>
+      </c>
+      <c r="E1166" t="s">
+        <v>3007</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1167" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1167" t="s">
+        <v>3008</v>
+      </c>
+      <c r="C1167" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D1167" t="s">
+        <v>3009</v>
+      </c>
+      <c r="E1167" t="s">
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1168" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1168" t="s">
+        <v>3011</v>
+      </c>
+      <c r="C1168" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D1168" t="s">
+        <v>3012</v>
+      </c>
+      <c r="E1168" t="s">
+        <v>3012</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1169" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1169" t="s">
+        <v>3013</v>
+      </c>
+      <c r="C1169" t="s">
+        <v>3014</v>
+      </c>
+      <c r="D1169" t="s">
+        <v>3015</v>
+      </c>
+      <c r="E1169" t="s">
+        <v>3016</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1170" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1170" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C1170" t="s">
+        <v>3018</v>
+      </c>
+      <c r="D1170" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E1170" t="s">
+        <v>3019</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1171" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1171" t="s">
+        <v>3020</v>
+      </c>
+      <c r="C1171" t="s">
+        <v>3021</v>
+      </c>
+      <c r="D1171" t="s">
+        <v>3021</v>
+      </c>
+      <c r="E1171" t="s">
+        <v>3022</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1172" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1172" t="s">
+        <v>3023</v>
+      </c>
+      <c r="C1172" t="s">
+        <v>3023</v>
+      </c>
+      <c r="D1172" t="s">
+        <v>3024</v>
+      </c>
+      <c r="E1172" t="s">
+        <v>3025</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1173" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1173" t="s">
+        <v>3026</v>
+      </c>
+      <c r="C1173" t="s">
+        <v>3026</v>
+      </c>
+      <c r="D1173" t="s">
+        <v>3027</v>
+      </c>
+      <c r="E1173" t="s">
+        <v>3028</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1174" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1174" t="s">
+        <v>3029</v>
+      </c>
+      <c r="C1174" t="s">
+        <v>3029</v>
+      </c>
+      <c r="D1174" t="s">
+        <v>3030</v>
+      </c>
+      <c r="E1174" t="s">
+        <v>3031</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1175" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1175" t="s">
+        <v>3032</v>
+      </c>
+      <c r="C1175" t="s">
+        <v>3032</v>
+      </c>
+      <c r="D1175" t="s">
+        <v>3032</v>
+      </c>
+      <c r="E1175" t="s">
+        <v>3033</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1176" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1176" t="s">
+        <v>3034</v>
+      </c>
+      <c r="C1176" t="s">
+        <v>3034</v>
+      </c>
+      <c r="D1176" t="s">
+        <v>3034</v>
+      </c>
+      <c r="E1176" t="s">
+        <v>3034</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1177" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1177" t="s">
+        <v>3035</v>
+      </c>
+      <c r="C1177" t="s">
+        <v>3036</v>
+      </c>
+      <c r="D1177" t="s">
+        <v>3036</v>
+      </c>
+      <c r="E1177" t="s">
+        <v>3037</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1178" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1178" t="s">
+        <v>3038</v>
+      </c>
+      <c r="C1178" t="s">
+        <v>3038</v>
+      </c>
+      <c r="D1178" t="s">
+        <v>3038</v>
+      </c>
+      <c r="E1178" t="s">
+        <v>3039</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1179" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1179" t="s">
+        <v>3040</v>
+      </c>
+      <c r="C1179" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D1179" t="s">
+        <v>3041</v>
+      </c>
+      <c r="E1179" t="s">
+        <v>3042</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1180" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1180" t="s">
+        <v>3043</v>
+      </c>
+      <c r="C1180" t="s">
+        <v>3044</v>
+      </c>
+      <c r="D1180" t="s">
+        <v>3044</v>
+      </c>
+      <c r="E1180" t="s">
+        <v>3045</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1181" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1181" t="s">
+        <v>3046</v>
+      </c>
+      <c r="C1181" t="s">
+        <v>3047</v>
+      </c>
+      <c r="D1181" t="s">
+        <v>3047</v>
+      </c>
+      <c r="E1181" t="s">
+        <v>3047</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1182" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1182" t="s">
+        <v>3048</v>
+      </c>
+      <c r="C1182" t="s">
+        <v>3048</v>
+      </c>
+      <c r="D1182" t="s">
+        <v>3049</v>
+      </c>
+      <c r="E1182" t="s">
+        <v>3050</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1183" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1183" t="s">
+        <v>3051</v>
+      </c>
+      <c r="C1183" t="s">
+        <v>3051</v>
+      </c>
+      <c r="D1183" t="s">
+        <v>3052</v>
+      </c>
+      <c r="E1183" t="s">
+        <v>3053</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1184" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1184" t="s">
+        <v>3054</v>
+      </c>
+      <c r="C1184" t="s">
+        <v>3054</v>
+      </c>
+      <c r="D1184" t="s">
+        <v>3055</v>
+      </c>
+      <c r="E1184" t="s">
+        <v>3056</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1185" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1185" t="s">
+        <v>3057</v>
+      </c>
+      <c r="C1185" t="s">
+        <v>3058</v>
+      </c>
+      <c r="D1185" t="s">
+        <v>3058</v>
+      </c>
+      <c r="E1185" t="s">
+        <v>3059</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1186" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1186" t="s">
+        <v>3060</v>
+      </c>
+      <c r="C1186" t="s">
+        <v>3061</v>
+      </c>
+      <c r="D1186" t="s">
+        <v>3061</v>
+      </c>
+      <c r="E1186" t="s">
+        <v>3062</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1187" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1187" t="s">
+        <v>3063</v>
+      </c>
+      <c r="C1187" t="s">
+        <v>3064</v>
+      </c>
+      <c r="D1187" t="s">
+        <v>3064</v>
+      </c>
+      <c r="E1187" t="s">
+        <v>3064</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1188" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1188" t="s">
+        <v>3065</v>
+      </c>
+      <c r="C1188" t="s">
+        <v>3066</v>
+      </c>
+      <c r="D1188" t="s">
+        <v>3066</v>
+      </c>
+      <c r="E1188" t="s">
+        <v>3066</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1189" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1189" t="s">
+        <v>3067</v>
+      </c>
+      <c r="C1189" t="s">
+        <v>3068</v>
+      </c>
+      <c r="D1189" t="s">
+        <v>3068</v>
+      </c>
+      <c r="E1189" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1190" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1190" t="s">
+        <v>3070</v>
+      </c>
+      <c r="C1190" t="s">
+        <v>3071</v>
+      </c>
+      <c r="D1190" t="s">
+        <v>3071</v>
+      </c>
+      <c r="E1190" t="s">
+        <v>3072</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1191" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1191" t="s">
+        <v>3073</v>
+      </c>
+      <c r="C1191" t="s">
+        <v>3074</v>
+      </c>
+      <c r="D1191" t="s">
+        <v>3074</v>
+      </c>
+      <c r="E1191" t="s">
+        <v>3075</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1192" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1192" t="s">
+        <v>3076</v>
+      </c>
+      <c r="C1192" t="s">
+        <v>3077</v>
+      </c>
+      <c r="D1192" t="s">
+        <v>3077</v>
+      </c>
+      <c r="E1192" t="s">
+        <v>3078</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1193" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1193" t="s">
+        <v>3079</v>
+      </c>
+      <c r="C1193" t="s">
+        <v>3080</v>
+      </c>
+      <c r="D1193" t="s">
+        <v>3081</v>
+      </c>
+      <c r="E1193" t="s">
+        <v>3082</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1194" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1194" t="s">
+        <v>3083</v>
+      </c>
+      <c r="C1194" t="s">
+        <v>3083</v>
+      </c>
+      <c r="D1194" t="s">
+        <v>3083</v>
+      </c>
+      <c r="E1194" t="s">
+        <v>3083</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1195" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1195" t="s">
+        <v>3084</v>
+      </c>
+      <c r="C1195" t="s">
+        <v>3084</v>
+      </c>
+      <c r="D1195" t="s">
+        <v>3085</v>
+      </c>
+      <c r="E1195" t="s">
+        <v>3086</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1196" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1196" t="s">
+        <v>3087</v>
+      </c>
+      <c r="C1196" t="s">
+        <v>3088</v>
+      </c>
+      <c r="D1196" t="s">
+        <v>3088</v>
+      </c>
+      <c r="E1196" t="s">
+        <v>3089</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1197" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1197" t="s">
+        <v>3090</v>
+      </c>
+      <c r="C1197" t="s">
+        <v>3090</v>
+      </c>
+      <c r="D1197" t="s">
+        <v>3090</v>
+      </c>
+      <c r="E1197" t="s">
+        <v>3091</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1198" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1198" t="s">
+        <v>3092</v>
+      </c>
+      <c r="C1198" t="s">
+        <v>3092</v>
+      </c>
+      <c r="D1198" t="s">
+        <v>3092</v>
+      </c>
+      <c r="E1198" t="s">
+        <v>3093</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1199" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1199" t="s">
+        <v>3094</v>
+      </c>
+      <c r="C1199" t="s">
+        <v>3095</v>
+      </c>
+      <c r="D1199" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E1199" t="s">
+        <v>3095</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1200" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1200" t="s">
+        <v>3096</v>
+      </c>
+      <c r="C1200" t="s">
+        <v>3097</v>
+      </c>
+      <c r="D1200" t="s">
+        <v>3097</v>
+      </c>
+      <c r="E1200" t="s">
+        <v>3098</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1201" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1201" t="s">
+        <v>3099</v>
+      </c>
+      <c r="C1201" t="s">
+        <v>3100</v>
+      </c>
+      <c r="D1201" t="s">
+        <v>3100</v>
+      </c>
+      <c r="E1201" t="s">
+        <v>3100</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86498916-66BE-6B4D-802E-4A534836EDA3}">
+  <dimension ref="A1:D101"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2820</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2821</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2822</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2823</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2824</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2824</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2825</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2826</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2827</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2827</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2828</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>2829</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2829</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2830</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2831</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>2832</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2833</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2833</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2834</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>2835</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2835</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2836</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2837</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>2838</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2838</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2839</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2840</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>2841</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2841</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2841</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2842</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>2843</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2844</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2844</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>2846</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2847</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2847</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2847</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>2848</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2848</v>
+      </c>
+      <c r="C11" t="s">
+        <v>2848</v>
+      </c>
+      <c r="D11" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>2849</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2850</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2851</v>
+      </c>
+      <c r="D12" t="s">
+        <v>2852</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>2853</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2853</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2854</v>
+      </c>
+      <c r="D13" t="s">
+        <v>2855</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>2856</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2856</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2857</v>
+      </c>
+      <c r="D14" t="s">
+        <v>2858</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>2859</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2859</v>
+      </c>
+      <c r="C15" t="s">
+        <v>2860</v>
+      </c>
+      <c r="D15" t="s">
+        <v>2861</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>2862</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2862</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2863</v>
+      </c>
+      <c r="D16" t="s">
+        <v>2864</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>2865</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2865</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2866</v>
+      </c>
+      <c r="D17" t="s">
+        <v>2867</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>2868</v>
+      </c>
+      <c r="B18" t="s">
+        <v>2868</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2869</v>
+      </c>
+      <c r="D18" t="s">
+        <v>2870</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>2871</v>
+      </c>
+      <c r="B19" t="s">
+        <v>2871</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2872</v>
+      </c>
+      <c r="D19" t="s">
+        <v>2873</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>2874</v>
+      </c>
+      <c r="B20" t="s">
+        <v>2874</v>
+      </c>
+      <c r="C20" t="s">
+        <v>2875</v>
+      </c>
+      <c r="D20" t="s">
+        <v>2876</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>2877</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2878</v>
+      </c>
+      <c r="C21" t="s">
+        <v>2878</v>
+      </c>
+      <c r="D21" t="s">
+        <v>2878</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>2879</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2880</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2880</v>
+      </c>
+      <c r="D22" t="s">
+        <v>2881</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>2882</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2883</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2883</v>
+      </c>
+      <c r="D23" t="s">
+        <v>2883</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>2884</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2885</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2885</v>
+      </c>
+      <c r="D24" t="s">
+        <v>2886</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>2887</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2888</v>
+      </c>
+      <c r="C25" t="s">
+        <v>2889</v>
+      </c>
+      <c r="D25" t="s">
+        <v>2890</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>2891</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2892</v>
+      </c>
+      <c r="C26" t="s">
+        <v>2893</v>
+      </c>
+      <c r="D26" t="s">
+        <v>2894</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>2895</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2896</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2897</v>
+      </c>
+      <c r="D27" t="s">
+        <v>2898</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>2899</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2900</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2900</v>
+      </c>
+      <c r="D28" t="s">
+        <v>2901</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>2902</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2903</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2903</v>
+      </c>
+      <c r="D29" t="s">
+        <v>2904</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>2905</v>
+      </c>
+      <c r="B30" t="s">
+        <v>2906</v>
+      </c>
+      <c r="C30" t="s">
+        <v>2907</v>
+      </c>
+      <c r="D30" t="s">
+        <v>2908</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>2909</v>
+      </c>
+      <c r="B31" t="s">
+        <v>2910</v>
+      </c>
+      <c r="C31" t="s">
+        <v>2911</v>
+      </c>
+      <c r="D31" t="s">
+        <v>2912</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>2913</v>
+      </c>
+      <c r="B32" t="s">
+        <v>2914</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2915</v>
+      </c>
+      <c r="D32" t="s">
+        <v>2916</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>2917</v>
+      </c>
+      <c r="B33" t="s">
+        <v>2918</v>
+      </c>
+      <c r="C33" t="s">
+        <v>2919</v>
+      </c>
+      <c r="D33" t="s">
+        <v>2920</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>2921</v>
+      </c>
+      <c r="B34" t="s">
+        <v>2922</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2923</v>
+      </c>
+      <c r="D34" t="s">
+        <v>2924</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>2925</v>
+      </c>
+      <c r="B35" t="s">
+        <v>2926</v>
+      </c>
+      <c r="C35" t="s">
+        <v>2927</v>
+      </c>
+      <c r="D35" t="s">
+        <v>2928</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>2929</v>
+      </c>
+      <c r="B36" t="s">
+        <v>2930</v>
+      </c>
+      <c r="C36" t="s">
+        <v>2930</v>
+      </c>
+      <c r="D36" t="s">
+        <v>2930</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>2931</v>
+      </c>
+      <c r="B37" t="s">
+        <v>2932</v>
+      </c>
+      <c r="C37" t="s">
+        <v>2932</v>
+      </c>
+      <c r="D37" t="s">
+        <v>2933</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>2934</v>
+      </c>
+      <c r="B38" t="s">
+        <v>2935</v>
+      </c>
+      <c r="C38" t="s">
+        <v>2935</v>
+      </c>
+      <c r="D38" t="s">
+        <v>2935</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>2936</v>
+      </c>
+      <c r="B39" t="s">
+        <v>2937</v>
+      </c>
+      <c r="C39" t="s">
+        <v>2937</v>
+      </c>
+      <c r="D39" t="s">
+        <v>2937</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>2938</v>
+      </c>
+      <c r="B40" t="s">
+        <v>2939</v>
+      </c>
+      <c r="C40" t="s">
+        <v>2939</v>
+      </c>
+      <c r="D40" t="s">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>2941</v>
+      </c>
+      <c r="B41" t="s">
+        <v>2942</v>
+      </c>
+      <c r="C41" t="s">
+        <v>2942</v>
+      </c>
+      <c r="D41" t="s">
+        <v>2943</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>2944</v>
+      </c>
+      <c r="B42" t="s">
+        <v>2944</v>
+      </c>
+      <c r="C42" t="s">
+        <v>2945</v>
+      </c>
+      <c r="D42" t="s">
+        <v>2946</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>2947</v>
+      </c>
+      <c r="B43" t="s">
+        <v>2948</v>
+      </c>
+      <c r="C43" t="s">
+        <v>2948</v>
+      </c>
+      <c r="D43" t="s">
+        <v>2949</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>2950</v>
+      </c>
+      <c r="B44" t="s">
+        <v>2951</v>
+      </c>
+      <c r="C44" t="s">
+        <v>2951</v>
+      </c>
+      <c r="D44" t="s">
+        <v>2952</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>2953</v>
+      </c>
+      <c r="B45" t="s">
+        <v>1753</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1753</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1753</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>2954</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1756</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1756</v>
+      </c>
+      <c r="D46" t="s">
+        <v>2955</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>2956</v>
+      </c>
+      <c r="B47" t="s">
+        <v>2957</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2957</v>
+      </c>
+      <c r="D47" t="s">
+        <v>2958</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>2959</v>
+      </c>
+      <c r="B48" t="s">
+        <v>2960</v>
+      </c>
+      <c r="C48" t="s">
+        <v>2960</v>
+      </c>
+      <c r="D48" t="s">
+        <v>2960</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>2961</v>
+      </c>
+      <c r="B49" t="s">
+        <v>2962</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2962</v>
+      </c>
+      <c r="D49" t="s">
+        <v>2962</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>2963</v>
+      </c>
+      <c r="B50" t="s">
+        <v>2964</v>
+      </c>
+      <c r="C50" t="s">
+        <v>2964</v>
+      </c>
+      <c r="D50" t="s">
+        <v>2965</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>2966</v>
+      </c>
+      <c r="B51" t="s">
+        <v>2967</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2967</v>
+      </c>
+      <c r="D51" t="s">
+        <v>2968</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>2969</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2969</v>
+      </c>
+      <c r="C52" t="s">
+        <v>2969</v>
+      </c>
+      <c r="D52" t="s">
+        <v>2969</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>2970</v>
+      </c>
+      <c r="B53" t="s">
+        <v>2971</v>
+      </c>
+      <c r="C53" t="s">
+        <v>2971</v>
+      </c>
+      <c r="D53" t="s">
+        <v>2971</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>2972</v>
+      </c>
+      <c r="B54" t="s">
+        <v>2973</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2973</v>
+      </c>
+      <c r="D54" t="s">
+        <v>2973</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>2974</v>
+      </c>
+      <c r="B55" t="s">
+        <v>2975</v>
+      </c>
+      <c r="C55" t="s">
+        <v>2975</v>
+      </c>
+      <c r="D55" t="s">
+        <v>2976</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>2977</v>
+      </c>
+      <c r="B56" t="s">
+        <v>2978</v>
+      </c>
+      <c r="C56" t="s">
+        <v>2978</v>
+      </c>
+      <c r="D56" t="s">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>2980</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2981</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2981</v>
+      </c>
+      <c r="D57" t="s">
+        <v>2982</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>2983</v>
+      </c>
+      <c r="B58" t="s">
+        <v>2984</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2985</v>
+      </c>
+      <c r="D58" t="s">
+        <v>2984</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>2986</v>
+      </c>
+      <c r="B59" t="s">
+        <v>2987</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2987</v>
+      </c>
+      <c r="D59" t="s">
+        <v>2987</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>2988</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2989</v>
+      </c>
+      <c r="C60" t="s">
+        <v>2989</v>
+      </c>
+      <c r="D60" t="s">
+        <v>2989</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>2990</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2991</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2992</v>
+      </c>
+      <c r="D61" t="s">
+        <v>2993</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>2994</v>
+      </c>
+      <c r="B62" t="s">
+        <v>2995</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2995</v>
+      </c>
+      <c r="D62" t="s">
+        <v>2996</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>583</v>
+      </c>
+      <c r="B63" t="s">
+        <v>2997</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2997</v>
+      </c>
+      <c r="D63" t="s">
+        <v>2997</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>2998</v>
+      </c>
+      <c r="B64" t="s">
+        <v>2999</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2999</v>
+      </c>
+      <c r="D64" t="s">
+        <v>2999</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>3000</v>
+      </c>
+      <c r="B65" t="s">
+        <v>3001</v>
+      </c>
+      <c r="C65" t="s">
+        <v>3002</v>
+      </c>
+      <c r="D65" t="s">
+        <v>3003</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>3004</v>
+      </c>
+      <c r="B66" t="s">
+        <v>3005</v>
+      </c>
+      <c r="C66" t="s">
+        <v>3006</v>
+      </c>
+      <c r="D66" t="s">
+        <v>3007</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>3008</v>
+      </c>
+      <c r="B67" t="s">
+        <v>3009</v>
+      </c>
+      <c r="C67" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D67" t="s">
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>3011</v>
+      </c>
+      <c r="B68" t="s">
+        <v>3012</v>
+      </c>
+      <c r="C68" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D68" t="s">
+        <v>3012</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>3013</v>
+      </c>
+      <c r="B69" t="s">
+        <v>3014</v>
+      </c>
+      <c r="C69" t="s">
+        <v>3015</v>
+      </c>
+      <c r="D69" t="s">
+        <v>3016</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>3017</v>
+      </c>
+      <c r="B70" t="s">
+        <v>3018</v>
+      </c>
+      <c r="C70" t="s">
+        <v>3018</v>
+      </c>
+      <c r="D70" t="s">
+        <v>3019</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>3020</v>
+      </c>
+      <c r="B71" t="s">
+        <v>3021</v>
+      </c>
+      <c r="C71" t="s">
+        <v>3021</v>
+      </c>
+      <c r="D71" t="s">
+        <v>3022</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>3023</v>
+      </c>
+      <c r="B72" t="s">
+        <v>3023</v>
+      </c>
+      <c r="C72" t="s">
+        <v>3024</v>
+      </c>
+      <c r="D72" t="s">
+        <v>3025</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>3026</v>
+      </c>
+      <c r="B73" t="s">
+        <v>3026</v>
+      </c>
+      <c r="C73" t="s">
+        <v>3027</v>
+      </c>
+      <c r="D73" t="s">
+        <v>3028</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>3029</v>
+      </c>
+      <c r="B74" t="s">
+        <v>3029</v>
+      </c>
+      <c r="C74" t="s">
+        <v>3030</v>
+      </c>
+      <c r="D74" t="s">
+        <v>3031</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>3032</v>
+      </c>
+      <c r="B75" t="s">
+        <v>3032</v>
+      </c>
+      <c r="C75" t="s">
+        <v>3032</v>
+      </c>
+      <c r="D75" t="s">
+        <v>3033</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>3034</v>
+      </c>
+      <c r="B76" t="s">
+        <v>3034</v>
+      </c>
+      <c r="C76" t="s">
+        <v>3034</v>
+      </c>
+      <c r="D76" t="s">
+        <v>3034</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>3035</v>
+      </c>
+      <c r="B77" t="s">
+        <v>3036</v>
+      </c>
+      <c r="C77" t="s">
+        <v>3036</v>
+      </c>
+      <c r="D77" t="s">
+        <v>3037</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>3038</v>
+      </c>
+      <c r="B78" t="s">
+        <v>3038</v>
+      </c>
+      <c r="C78" t="s">
+        <v>3038</v>
+      </c>
+      <c r="D78" t="s">
+        <v>3039</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>3040</v>
+      </c>
+      <c r="B79" t="s">
+        <v>3041</v>
+      </c>
+      <c r="C79" t="s">
+        <v>3041</v>
+      </c>
+      <c r="D79" t="s">
+        <v>3042</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>3043</v>
+      </c>
+      <c r="B80" t="s">
+        <v>3044</v>
+      </c>
+      <c r="C80" t="s">
+        <v>3044</v>
+      </c>
+      <c r="D80" t="s">
+        <v>3045</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>3046</v>
+      </c>
+      <c r="B81" t="s">
+        <v>3047</v>
+      </c>
+      <c r="C81" t="s">
+        <v>3047</v>
+      </c>
+      <c r="D81" t="s">
+        <v>3047</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>3048</v>
+      </c>
+      <c r="B82" t="s">
+        <v>3048</v>
+      </c>
+      <c r="C82" t="s">
+        <v>3049</v>
+      </c>
+      <c r="D82" t="s">
+        <v>3050</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>3051</v>
+      </c>
+      <c r="B83" t="s">
+        <v>3051</v>
+      </c>
+      <c r="C83" t="s">
+        <v>3052</v>
+      </c>
+      <c r="D83" t="s">
+        <v>3053</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>3054</v>
+      </c>
+      <c r="B84" t="s">
+        <v>3054</v>
+      </c>
+      <c r="C84" t="s">
+        <v>3055</v>
+      </c>
+      <c r="D84" t="s">
+        <v>3056</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>3057</v>
+      </c>
+      <c r="B85" t="s">
+        <v>3058</v>
+      </c>
+      <c r="C85" t="s">
+        <v>3058</v>
+      </c>
+      <c r="D85" t="s">
+        <v>3059</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>3060</v>
+      </c>
+      <c r="B86" t="s">
+        <v>3061</v>
+      </c>
+      <c r="C86" t="s">
+        <v>3061</v>
+      </c>
+      <c r="D86" t="s">
+        <v>3062</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>3063</v>
+      </c>
+      <c r="B87" t="s">
+        <v>3064</v>
+      </c>
+      <c r="C87" t="s">
+        <v>3064</v>
+      </c>
+      <c r="D87" t="s">
+        <v>3064</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>3065</v>
+      </c>
+      <c r="B88" t="s">
+        <v>3066</v>
+      </c>
+      <c r="C88" t="s">
+        <v>3066</v>
+      </c>
+      <c r="D88" t="s">
+        <v>3066</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>3067</v>
+      </c>
+      <c r="B89" t="s">
+        <v>3068</v>
+      </c>
+      <c r="C89" t="s">
+        <v>3068</v>
+      </c>
+      <c r="D89" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>3070</v>
+      </c>
+      <c r="B90" t="s">
+        <v>3071</v>
+      </c>
+      <c r="C90" t="s">
+        <v>3071</v>
+      </c>
+      <c r="D90" t="s">
+        <v>3072</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>3073</v>
+      </c>
+      <c r="B91" t="s">
+        <v>3074</v>
+      </c>
+      <c r="C91" t="s">
+        <v>3074</v>
+      </c>
+      <c r="D91" t="s">
+        <v>3075</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>3076</v>
+      </c>
+      <c r="B92" t="s">
+        <v>3077</v>
+      </c>
+      <c r="C92" t="s">
+        <v>3077</v>
+      </c>
+      <c r="D92" t="s">
+        <v>3078</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>3079</v>
+      </c>
+      <c r="B93" t="s">
+        <v>3080</v>
+      </c>
+      <c r="C93" t="s">
+        <v>3081</v>
+      </c>
+      <c r="D93" t="s">
+        <v>3082</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>3083</v>
+      </c>
+      <c r="B94" t="s">
+        <v>3083</v>
+      </c>
+      <c r="C94" t="s">
+        <v>3083</v>
+      </c>
+      <c r="D94" t="s">
+        <v>3083</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>3084</v>
+      </c>
+      <c r="B95" t="s">
+        <v>3084</v>
+      </c>
+      <c r="C95" t="s">
+        <v>3085</v>
+      </c>
+      <c r="D95" t="s">
+        <v>3086</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>3087</v>
+      </c>
+      <c r="B96" t="s">
+        <v>3088</v>
+      </c>
+      <c r="C96" t="s">
+        <v>3088</v>
+      </c>
+      <c r="D96" t="s">
+        <v>3089</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>3090</v>
+      </c>
+      <c r="B97" t="s">
+        <v>3090</v>
+      </c>
+      <c r="C97" t="s">
+        <v>3090</v>
+      </c>
+      <c r="D97" t="s">
+        <v>3091</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>3092</v>
+      </c>
+      <c r="B98" t="s">
+        <v>3092</v>
+      </c>
+      <c r="C98" t="s">
+        <v>3092</v>
+      </c>
+      <c r="D98" t="s">
+        <v>3093</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>3094</v>
+      </c>
+      <c r="B99" t="s">
+        <v>3095</v>
+      </c>
+      <c r="C99" t="s">
+        <v>3095</v>
+      </c>
+      <c r="D99" t="s">
+        <v>3095</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>3096</v>
+      </c>
+      <c r="B100" t="s">
+        <v>3097</v>
+      </c>
+      <c r="C100" t="s">
+        <v>3097</v>
+      </c>
+      <c r="D100" t="s">
+        <v>3098</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>3099</v>
+      </c>
+      <c r="B101" t="s">
+        <v>3100</v>
+      </c>
+      <c r="C101" t="s">
+        <v>3100</v>
+      </c>
+      <c r="D101" t="s">
+        <v>3100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>